<commit_message>
Working along; no real updates. Sorry future me.
</commit_message>
<xml_diff>
--- a/WorkBot/main/data/orders/Ithaca Bakery/combined_orders_Ithaca Bakery.xlsx
+++ b/WorkBot/main/data/orders/Ithaca Bakery/combined_orders_Ithaca Bakery.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andrew\Desktop\Andrew\Projects\IthacaBakery\RandomStuff\WorkBot\main\data\orders\Ithaca Bakery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B06B3857-42B8-4E98-90A0-01946299DA07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4B7B57B-631C-4F4C-86A5-608B688701E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,12 +18,23 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Sheet!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="122">
   <si>
     <t>Item Name</t>
   </si>
@@ -49,10 +60,10 @@
     <t>Bag Paper - Baguette</t>
   </si>
   <si>
-    <t>Bindi - Cake Tiramisu Round</t>
-  </si>
-  <si>
-    <t>Can - Coconut Milk</t>
+    <t>Box Cake - 8x8x5</t>
+  </si>
+  <si>
+    <t>Cake - Tres Leches</t>
   </si>
   <si>
     <t>Capers</t>
@@ -70,13 +81,13 @@
     <t>Chobani - Drinkables (Protein, Assorted)</t>
   </si>
   <si>
-    <t>Coconut - Sweet Flake</t>
+    <t>Coffee Stirrer (Bamboo)</t>
   </si>
   <si>
     <t>Container - Deli (16oz)</t>
   </si>
   <si>
-    <t>Container - Muffin (1 Pack)</t>
+    <t>Container - Deli (8oz)</t>
   </si>
   <si>
     <t>Container - Plastic Clamshell (6")</t>
@@ -88,24 +99,78 @@
     <t>Container - Soup (8oz)</t>
   </si>
   <si>
-    <t>Copy Paper (8.5" x 11")</t>
-  </si>
-  <si>
     <t>Cup - Espresso (4oz)</t>
   </si>
   <si>
     <t>Cup - Hot (8oz)</t>
   </si>
   <si>
+    <t>Cup - Portion (2oz)</t>
+  </si>
+  <si>
+    <t>Cup - Portion (3.25oz)</t>
+  </si>
+  <si>
+    <t>DV - Butter Toffee Almonds (bulk)</t>
+  </si>
+  <si>
+    <t>DV - Caramel Lovers Dream (bulk)</t>
+  </si>
+  <si>
+    <t>DV - Cheddar Lovers Snack Mix (bulk)</t>
+  </si>
+  <si>
+    <t>DV - Chocolate Mini Pretzel</t>
+  </si>
+  <si>
+    <t>DV - Dk Choc Rasp Cup (bulk)</t>
+  </si>
+  <si>
+    <t>DV - Gummi Bears (8 oz)</t>
+  </si>
+  <si>
+    <t>DV - Gummi Peach Rings</t>
+  </si>
+  <si>
+    <t>DV - Gummi Sharks</t>
+  </si>
+  <si>
+    <t>DV - Licorice Allsort</t>
+  </si>
+  <si>
+    <t>DV - Milk Caramel Peanut Cluster (bulk)</t>
+  </si>
+  <si>
+    <t>DV - Orange Slices</t>
+  </si>
+  <si>
+    <t>DV - PB filled Pretzels (bulk)</t>
+  </si>
+  <si>
+    <t>DV - PB&amp;J Snack Mix (bulk)</t>
+  </si>
+  <si>
+    <t>DV - Real Fruit Sour Bursts (bulk)</t>
+  </si>
+  <si>
+    <t>DV - Sesame Stx Honey Roast (bulk)</t>
+  </si>
+  <si>
+    <t>DV - Sour Neon Gummi Worms</t>
+  </si>
+  <si>
+    <t>DV - Watermelon Chamoy Gummie Ring (bulk)</t>
+  </si>
+  <si>
+    <t>DV - Yogurt Covered Raisins (bulk)</t>
+  </si>
+  <si>
     <t>Degreaser - for Panini Press (Dawn)</t>
   </si>
   <si>
     <t>Egg Patty - Vegan</t>
   </si>
   <si>
-    <t>Eggs (In-Shell)</t>
-  </si>
-  <si>
     <t>Employee Water</t>
   </si>
   <si>
@@ -118,22 +183,22 @@
     <t>FRZ Fruit - Mango</t>
   </si>
   <si>
-    <t>FRZ Fruit - Raspberry (Whole)</t>
-  </si>
-  <si>
     <t>Fiji Water 1L</t>
   </si>
   <si>
     <t>Fiji Water 500ml</t>
   </si>
   <si>
-    <t>Flax Seeds</t>
-  </si>
-  <si>
     <t>Floor Cleaner - Lucky 7</t>
   </si>
   <si>
-    <t>Flour - Millers Choice</t>
+    <t>Garlic Spread</t>
+  </si>
+  <si>
+    <t>Goat Cheese</t>
+  </si>
+  <si>
+    <t>Grandma's Coffee Cake - Apple</t>
   </si>
   <si>
     <t>Grandma's Coffee Cake - Banana Walnut</t>
@@ -142,13 +207,13 @@
     <t>Grandma's Coffee Cake - Blueberry</t>
   </si>
   <si>
+    <t>Grandma's Coffee Cake - Chocolate Chip</t>
+  </si>
+  <si>
     <t>Grandma's Coffee Cake - Chocolate Walnut</t>
   </si>
   <si>
-    <t>Grandma's Coffee Cake - Cinnamon w/ Nuts</t>
-  </si>
-  <si>
-    <t>Grandma's Coffee Cake - Cranberry</t>
+    <t>Grandma's Coffee Cake - Cinnamon</t>
   </si>
   <si>
     <t>Grandma's Coffee Cake - Mixed Berry</t>
@@ -160,64 +225,70 @@
     <t>Honey - Jug</t>
   </si>
   <si>
+    <t>Hot Chocolate (Bulk)</t>
+  </si>
+  <si>
+    <t>Iced Tea - Green Citrus Ginko</t>
+  </si>
+  <si>
+    <t>Ithaca Soda - Ginger Beer</t>
+  </si>
+  <si>
+    <t>Ithaca Soda - Root Beer</t>
+  </si>
+  <si>
     <t>Java Box (160oz)</t>
   </si>
   <si>
-    <t>Java Box (96oz)</t>
-  </si>
-  <si>
-    <t>Jelly - Grape</t>
-  </si>
-  <si>
     <t>Joe Tea - Black Cherry</t>
   </si>
   <si>
-    <t>Joe Tea - Classic Lemonade</t>
-  </si>
-  <si>
-    <t>Joe Tea - Kiwi Strawberry</t>
+    <t>Joe Tea - Raspberry</t>
+  </si>
+  <si>
+    <t>Key Chain Bottle Opener</t>
   </si>
   <si>
     <t>Kilogram Chai Concentrate</t>
   </si>
   <si>
+    <t>Koozie - Ib</t>
+  </si>
+  <si>
     <t>Lid - Deli (6/32oz)</t>
   </si>
   <si>
-    <t>Lid - Hot Cup (8oz)</t>
+    <t>Lid - Portion (2oz)</t>
   </si>
   <si>
     <t>Lid - Portion (3.25oz)</t>
   </si>
   <si>
-    <t>Lid - Soup (32oz)</t>
-  </si>
-  <si>
     <t>Lid - Soup (6/16 oz)</t>
   </si>
   <si>
+    <t>Lid Espresso - 4oz</t>
+  </si>
+  <si>
+    <t>Long Sleeve Shirt - Dog w/ Baguette</t>
+  </si>
+  <si>
     <t>Maple Syrup (pure)</t>
   </si>
   <si>
     <t>Matcha</t>
   </si>
   <si>
-    <t>Monin - Cinnamon</t>
-  </si>
-  <si>
     <t>Monin - Guava Puree</t>
   </si>
   <si>
-    <t>Mop Head Cut (White)</t>
-  </si>
-  <si>
-    <t>Non-Dairy Creamer</t>
-  </si>
-  <si>
-    <t>Oats</t>
-  </si>
-  <si>
-    <t>Oil - Olive Extra Virgin</t>
+    <t>Monin - Spiced Brown Sugar</t>
+  </si>
+  <si>
+    <t>Mug - Stoneware Pottery (java taster)</t>
+  </si>
+  <si>
+    <t>Peanut Butter - Chunky</t>
   </si>
   <si>
     <t>Peanut Butter - Creamy</t>
@@ -229,30 +300,36 @@
     <t>Red Bull - Amber</t>
   </si>
   <si>
-    <t>Register Tape - Thermal (3.125" x 230')</t>
-  </si>
-  <si>
     <t>Saratoga Sparkling 12oz</t>
   </si>
   <si>
+    <t>Saratoga Sparkling 28oz</t>
+  </si>
+  <si>
+    <t>Scrubbies - Steel</t>
+  </si>
+  <si>
     <t>Smoked Salmon (Retail Pack)</t>
   </si>
   <si>
-    <t>Smoked Salmon (Sliced)</t>
-  </si>
-  <si>
-    <t>Sugar - Light Brown</t>
+    <t>Supplement - Antioxident</t>
   </si>
   <si>
     <t>Supplement - Collagen</t>
   </si>
   <si>
-    <t>Supplement - Hangover</t>
-  </si>
-  <si>
     <t>Supplement - Whey Protein</t>
   </si>
   <si>
+    <t>Sweatshirt Dog w/ Bagel (crew neck)</t>
+  </si>
+  <si>
+    <t>Sweatshirt Pullover - Baked in Ithaca (hoodie)</t>
+  </si>
+  <si>
+    <t>Sweatshirt Pullover - SYR Logo (hoodie)</t>
+  </si>
+  <si>
     <t>Sweet Street - Bar Lemon Luscious Sliced</t>
   </si>
   <si>
@@ -262,12 +339,12 @@
     <t>Sweet Street - Chocolate Lovin</t>
   </si>
   <si>
-    <t>Sweet Street - Pie Choc PB Cup Sliced</t>
-  </si>
-  <si>
     <t>Sweet Street - Pie Oreo Cookie Bash Sliced</t>
   </si>
   <si>
+    <t>T- Shirt - Syr Logo</t>
+  </si>
+  <si>
     <t>Tea Bags - Earl Grey (Twinings)</t>
   </si>
   <si>
@@ -280,7 +357,7 @@
     <t>Tea Bags - Lemon Ginger (Twinings)</t>
   </si>
   <si>
-    <t>Tea Bags - Pomegrantate &amp; Rasp (Twinings)</t>
+    <t>Tea Towel - Coffee</t>
   </si>
   <si>
     <t>Torani - Caramel Sauce</t>
@@ -292,12 +369,15 @@
     <t>Torani - White Chocolate Sauce</t>
   </si>
   <si>
+    <t>Tote Bag - Mini (baked in ithaca)</t>
+  </si>
+  <si>
+    <t>Turbo Chef - Oven Cleaning Kit</t>
+  </si>
+  <si>
     <t>Urnex - Cafiza</t>
   </si>
   <si>
-    <t>Urnex - Grindz</t>
-  </si>
-  <si>
     <t>Urnex - Rinza</t>
   </si>
   <si>
@@ -317,6 +397,9 @@
   </si>
   <si>
     <t>Wrap - Paper (6" x 10.75")</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -760,12 +843,12 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E94"/>
+  <dimension ref="A1:E118"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="53.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="15.42578125" style="5" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" style="6" customWidth="1"/>
+    <col min="2" max="4" width="16.5703125" style="5" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -801,7 +884,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -811,33 +894,30 @@
       <c r="D4" s="5">
         <v>2</v>
       </c>
-      <c r="E4" s="6">
-        <v>2</v>
-      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="5">
-        <v>2</v>
+      <c r="C5" s="5">
+        <v>1</v>
       </c>
       <c r="D5" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="6">
-        <v>1</v>
-      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>10</v>
       </c>
+      <c r="C7" s="5">
+        <v>3</v>
+      </c>
       <c r="D7" s="5">
         <v>1</v>
       </c>
@@ -846,29 +926,32 @@
       <c r="A8" s="4" t="s">
         <v>11</v>
       </c>
+      <c r="B8" s="5">
+        <v>2</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>12</v>
       </c>
+      <c r="B9" s="5">
+        <v>2</v>
+      </c>
       <c r="C9" s="5">
         <v>2</v>
       </c>
       <c r="D9" s="5">
         <v>1</v>
-      </c>
-      <c r="E9" s="6">
-        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
+      <c r="B10" s="5">
+        <v>2</v>
+      </c>
       <c r="D10" s="5">
-        <v>1</v>
-      </c>
-      <c r="E10" s="6">
         <v>1</v>
       </c>
     </row>
@@ -876,7 +959,13 @@
       <c r="A11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="6">
+      <c r="B11" s="5">
+        <v>2</v>
+      </c>
+      <c r="C11" s="5">
+        <v>1</v>
+      </c>
+      <c r="D11" s="5">
         <v>1</v>
       </c>
     </row>
@@ -884,7 +973,7 @@
       <c r="A12" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="6">
+      <c r="B12" s="5">
         <v>1</v>
       </c>
     </row>
@@ -892,14 +981,8 @@
       <c r="A13" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="5">
-        <v>3</v>
-      </c>
-      <c r="C13" s="5">
-        <v>1</v>
-      </c>
       <c r="D13" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -909,6 +992,9 @@
       <c r="C14" s="5">
         <v>1</v>
       </c>
+      <c r="D14" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
@@ -917,22 +1003,19 @@
       <c r="B15" s="5">
         <v>1</v>
       </c>
-      <c r="C15" s="5">
-        <v>1</v>
-      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B16" s="5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C16" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" s="5">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -940,20 +1023,26 @@
         <v>20</v>
       </c>
       <c r="B17" s="5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C17" s="5">
         <v>1</v>
       </c>
       <c r="D17" s="5">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>21</v>
       </c>
+      <c r="B18" s="5">
+        <v>1</v>
+      </c>
       <c r="C18" s="5">
+        <v>1</v>
+      </c>
+      <c r="D18" s="5">
         <v>1</v>
       </c>
     </row>
@@ -961,19 +1050,19 @@
       <c r="A19" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="5">
-        <v>1</v>
+      <c r="C19" s="5">
+        <v>1</v>
+      </c>
+      <c r="D19" s="5">
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B20" s="5">
-        <v>12</v>
-      </c>
       <c r="D20" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -983,16 +1072,13 @@
       <c r="B21" s="5">
         <v>1</v>
       </c>
-      <c r="D21" s="5">
-        <v>1</v>
-      </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>25</v>
       </c>
       <c r="E22" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
@@ -1000,132 +1086,99 @@
         <v>26</v>
       </c>
       <c r="E23" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="5">
-        <v>2</v>
-      </c>
-      <c r="D24" s="5">
-        <v>3</v>
-      </c>
       <c r="E24" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D25" s="5">
-        <v>1</v>
+      <c r="E25" s="6">
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C26" s="5">
-        <v>2</v>
-      </c>
-      <c r="D26" s="5">
-        <v>1</v>
+      <c r="B26" s="5">
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B27" s="5">
-        <v>1</v>
-      </c>
       <c r="E27" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="5">
-        <v>1</v>
+      <c r="E28" s="6">
+        <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C29" s="5">
-        <v>1</v>
-      </c>
-      <c r="D29" s="5">
-        <v>1</v>
-      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D30" s="5">
-        <v>1</v>
-      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>34</v>
       </c>
       <c r="B31" s="5">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="5">
-        <v>1</v>
+      <c r="E32" s="6">
+        <v>4</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E33" s="6">
-        <v>1</v>
-      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="5">
-        <v>1</v>
-      </c>
-      <c r="E34" s="6">
-        <v>1</v>
-      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D35" s="5">
-        <v>1</v>
-      </c>
-      <c r="E35" s="6">
-        <v>2</v>
+      <c r="B35" s="5">
+        <v>6</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E36" s="6">
-        <v>2</v>
+      <c r="B36" s="5">
+        <v>6</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
@@ -1133,7 +1186,10 @@
         <v>40</v>
       </c>
       <c r="B37" s="5">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="E37" s="6">
+        <v>4</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
@@ -1141,7 +1197,7 @@
         <v>41</v>
       </c>
       <c r="B38" s="5">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
@@ -1149,7 +1205,7 @@
         <v>42</v>
       </c>
       <c r="D39" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
@@ -1157,40 +1213,43 @@
         <v>43</v>
       </c>
       <c r="B40" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D40" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C41" s="5">
-        <v>1</v>
-      </c>
-      <c r="D41" s="5">
-        <v>2</v>
+      <c r="B41" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>45</v>
       </c>
+      <c r="C42" s="5">
+        <v>1</v>
+      </c>
+      <c r="D42" s="5">
+        <v>3</v>
+      </c>
       <c r="E42" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>46</v>
       </c>
+      <c r="C43" s="5">
+        <v>1</v>
+      </c>
       <c r="D43" s="5">
-        <v>1</v>
-      </c>
-      <c r="E43" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
@@ -1200,14 +1259,14 @@
       <c r="C44" s="5">
         <v>1</v>
       </c>
+      <c r="D44" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C45" s="5">
-        <v>1</v>
-      </c>
       <c r="D45" s="5">
         <v>1</v>
       </c>
@@ -1216,7 +1275,7 @@
       <c r="A46" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C46" s="5">
+      <c r="D46" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1224,22 +1283,19 @@
       <c r="A47" s="4" t="s">
         <v>50</v>
       </c>
+      <c r="C47" s="5">
+        <v>1</v>
+      </c>
+      <c r="D47" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>51</v>
       </c>
       <c r="B48" s="5">
-        <v>3</v>
-      </c>
-      <c r="C48" s="5">
-        <v>2</v>
-      </c>
-      <c r="D48" s="5">
-        <v>2</v>
-      </c>
-      <c r="E48" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
@@ -1247,12 +1303,6 @@
         <v>52</v>
       </c>
       <c r="B49" s="5">
-        <v>6</v>
-      </c>
-      <c r="C49" s="5">
-        <v>2</v>
-      </c>
-      <c r="D49" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1261,9 +1311,9 @@
         <v>53</v>
       </c>
       <c r="B50" s="5">
-        <v>2</v>
-      </c>
-      <c r="C50" s="5">
+        <v>5</v>
+      </c>
+      <c r="D50" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1271,9 +1321,6 @@
       <c r="A51" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B51" s="5">
-        <v>1</v>
-      </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
@@ -1288,28 +1335,25 @@
         <v>56</v>
       </c>
       <c r="B53" s="5">
-        <v>4</v>
-      </c>
-      <c r="C53" s="5">
-        <v>2</v>
-      </c>
-      <c r="D53" s="5">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="E53" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="E54" s="6">
-        <v>2</v>
+      <c r="B54" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C55" s="5">
+      <c r="E55" s="6">
         <v>1</v>
       </c>
     </row>
@@ -1317,13 +1361,19 @@
       <c r="A56" s="4" t="s">
         <v>59</v>
       </c>
+      <c r="D56" s="5">
+        <v>1</v>
+      </c>
+      <c r="E56" s="6">
+        <v>1</v>
+      </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
         <v>60</v>
       </c>
       <c r="D57" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
@@ -1331,17 +1381,20 @@
         <v>61</v>
       </c>
       <c r="B58" s="5">
-        <v>3</v>
+        <v>2</v>
+      </c>
+      <c r="C58" s="5">
+        <v>1</v>
       </c>
       <c r="D58" s="5">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C59" s="5">
+      <c r="D59" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1366,17 +1419,17 @@
         <v>65</v>
       </c>
       <c r="C62" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D62" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C63" s="5">
+      <c r="D63" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1384,6 +1437,9 @@
       <c r="A64" s="4" t="s">
         <v>67</v>
       </c>
+      <c r="D64" s="5">
+        <v>1</v>
+      </c>
       <c r="E64" s="6">
         <v>1</v>
       </c>
@@ -1395,53 +1451,59 @@
       <c r="B65" s="5">
         <v>1</v>
       </c>
+      <c r="C65" s="5">
+        <v>1</v>
+      </c>
+      <c r="D65" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="D66" s="5">
-        <v>2</v>
-      </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D67" s="5">
-        <v>1</v>
-      </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
         <v>71</v>
       </c>
+      <c r="B68" s="5">
+        <v>2</v>
+      </c>
+      <c r="C68" s="5">
+        <v>1</v>
+      </c>
       <c r="D68" s="5">
         <v>1</v>
       </c>
       <c r="E68" s="6">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="E69" s="6">
-        <v>1</v>
-      </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
         <v>73</v>
       </c>
+      <c r="D70" s="5">
+        <v>3</v>
+      </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
         <v>74</v>
       </c>
       <c r="D71" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
@@ -1459,31 +1521,34 @@
       <c r="A73" s="4" t="s">
         <v>76</v>
       </c>
+      <c r="C73" s="5">
+        <v>1</v>
+      </c>
       <c r="D73" s="5">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E74" s="6">
-        <v>2</v>
+      <c r="B74" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="E75" s="6">
-        <v>1</v>
+      <c r="D75" s="5">
+        <v>10</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B76" s="5">
+      <c r="D76" s="5">
         <v>1</v>
       </c>
       <c r="E76" s="6">
@@ -1494,76 +1559,76 @@
       <c r="A77" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="B77" s="5">
+      <c r="C77" s="5">
         <v>1</v>
       </c>
       <c r="D77" s="5">
         <v>1</v>
+      </c>
+      <c r="E77" s="6">
+        <v>4</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C78" s="5">
-        <v>1</v>
-      </c>
-      <c r="E78" s="6">
-        <v>6</v>
+      <c r="B78" s="5">
+        <v>2</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C79" s="5">
-        <v>2</v>
-      </c>
-      <c r="E79" s="6">
-        <v>6</v>
+      <c r="B79" s="5">
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="C80" s="5">
-        <v>1</v>
-      </c>
-      <c r="E80" s="6">
-        <v>6</v>
+      <c r="D80" s="5">
+        <v>4</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="E81" s="6">
-        <v>6</v>
+      <c r="B81" s="5">
+        <v>2</v>
+      </c>
+      <c r="C81" s="5">
+        <v>1</v>
+      </c>
+      <c r="D81" s="5">
+        <v>2</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>85</v>
       </c>
+      <c r="B82" s="5">
+        <v>1</v>
+      </c>
       <c r="C82" s="5">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D82" s="5">
+        <v>4</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B83" s="5">
-        <v>1</v>
-      </c>
       <c r="C83" s="5">
         <v>1</v>
       </c>
       <c r="D83" s="5">
-        <v>3</v>
-      </c>
-      <c r="E83" s="6">
         <v>1</v>
       </c>
     </row>
@@ -1571,24 +1636,18 @@
       <c r="A84" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B84" s="5">
-        <v>3</v>
-      </c>
       <c r="C84" s="5">
         <v>1</v>
       </c>
-      <c r="D84" s="5">
-        <v>6</v>
-      </c>
       <c r="E84" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="E85" s="6">
+      <c r="D85" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1596,12 +1655,15 @@
       <c r="A86" s="4" t="s">
         <v>89</v>
       </c>
+      <c r="B86" s="5">
+        <v>1</v>
+      </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="D87" s="5">
+      <c r="C87" s="5">
         <v>1</v>
       </c>
     </row>
@@ -1609,76 +1671,298 @@
       <c r="A88" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="C88" s="5">
-        <v>1</v>
+      <c r="D88" s="5">
+        <v>1</v>
+      </c>
+      <c r="E88" s="6">
+        <v>2</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
-        <v>92</v>
+        <v>121</v>
+      </c>
+      <c r="B89" s="5">
+        <v>7</v>
       </c>
       <c r="C89" s="5">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="D89" s="5">
+        <v>3</v>
+      </c>
+      <c r="E89" s="6">
+        <v>4</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D90" s="5">
+        <v>92</v>
+      </c>
+      <c r="C90" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D91" s="5">
+        <v>93</v>
+      </c>
+      <c r="C91" s="5">
         <v>1</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B92" s="5">
-        <v>4</v>
-      </c>
-      <c r="C92" s="5">
         <v>1</v>
       </c>
       <c r="D92" s="5">
-        <v>1</v>
-      </c>
-      <c r="E92" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B93" s="5">
-        <v>2</v>
-      </c>
-      <c r="C93" s="5">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="D93" s="5">
-        <v>2</v>
-      </c>
-      <c r="E93" s="6">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D94" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A95" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B94" s="5">
-        <v>1</v>
-      </c>
-      <c r="D94" s="5">
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A96" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D96" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A97" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D97" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A98" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B98" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A99" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D99" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A100" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A101" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C101" s="5">
+        <v>1</v>
+      </c>
+      <c r="D101" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A102" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C102" s="5">
+        <v>1</v>
+      </c>
+      <c r="D102" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A103" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C103" s="5">
+        <v>1</v>
+      </c>
+      <c r="D103" s="5">
+        <v>2</v>
+      </c>
+      <c r="E103" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A104" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A105" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D105" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A106" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B106" s="5">
+        <v>2</v>
+      </c>
+      <c r="C106" s="5">
+        <v>1</v>
+      </c>
+      <c r="D106" s="5">
+        <v>2</v>
+      </c>
+      <c r="E106" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A107" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B107" s="5">
+        <v>2</v>
+      </c>
+      <c r="C107" s="5">
+        <v>1</v>
+      </c>
+      <c r="D107" s="5">
+        <v>3</v>
+      </c>
+      <c r="E107" s="6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A108" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B108" s="5">
+        <v>2</v>
+      </c>
+      <c r="C108" s="5">
+        <v>1</v>
+      </c>
+      <c r="D108" s="5">
+        <v>1</v>
+      </c>
+      <c r="E108" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A109" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D109" s="5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A110" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B110" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A111" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C111" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A112" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C112" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A113" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D113" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A114" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D114" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A115" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="C115" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A116" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E116" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A117" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C117" s="5">
+        <v>1</v>
+      </c>
+      <c r="D117" s="5">
+        <v>1</v>
+      </c>
+      <c r="E117" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A118" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D118" s="5">
         <v>1</v>
       </c>
     </row>

</xml_diff>